<commit_message>
CCs and CFs writing to db. Code tidied
</commit_message>
<xml_diff>
--- a/input_files/batched_new_capacity.xlsx
+++ b/input_files/batched_new_capacity.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://utoronto-my.sharepoint.com/personal/ian_elder_mail_utoronto_ca/Documents/Documents/TEMOA/CODERS scripts/input_files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="28" documentId="11_F25DC773A252ABDACC104858199A58E65ADE58E8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A9B6428F-E453-4035-8F8C-84D82ED988C4}"/>
+  <xr:revisionPtr revIDLastSave="30" documentId="11_F25DC773A252ABDACC104858199A58E65ADE58E8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B11C2137-0FFE-4994-90CF-65A60F7A4120}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
     <t>Sets the capacity for batches of new installed capacity by technology. For updating assumptions by quantity of new capacity.</t>
   </si>
@@ -40,6 +40,9 @@
   </si>
   <si>
     <t>tech_generic</t>
+  </si>
+  <si>
+    <t>HYDRO_RUN</t>
   </si>
 </sst>
 </file>
@@ -357,7 +360,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K5"/>
+  <dimension ref="A1:K6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17.7109375" bestFit="1" customWidth="1"/>
@@ -478,6 +481,41 @@
         <v>1000</v>
       </c>
     </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>5</v>
+      </c>
+      <c r="B6">
+        <v>1000</v>
+      </c>
+      <c r="C6">
+        <v>1000</v>
+      </c>
+      <c r="D6">
+        <v>1000</v>
+      </c>
+      <c r="E6">
+        <v>1000</v>
+      </c>
+      <c r="F6">
+        <v>1000</v>
+      </c>
+      <c r="G6">
+        <v>1000</v>
+      </c>
+      <c r="H6">
+        <v>1000</v>
+      </c>
+      <c r="I6">
+        <v>1000</v>
+      </c>
+      <c r="J6">
+        <v>1000</v>
+      </c>
+      <c r="K6">
+        <v>1000</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Adjusted for a quirk in IESO generation data
</commit_message>
<xml_diff>
--- a/input_files/batched_new_capacity.xlsx
+++ b/input_files/batched_new_capacity.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://utoronto-my.sharepoint.com/personal/ian_elder_mail_utoronto_ca/Documents/Documents/TEMOA/CODERS scripts/input_files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="30" documentId="11_F25DC773A252ABDACC104858199A58E65ADE58E8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B11C2137-0FFE-4994-90CF-65A60F7A4120}"/>
+  <xr:revisionPtr revIDLastSave="31" documentId="11_F25DC773A252ABDACC104858199A58E65ADE58E8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DB8E628F-AAAD-448E-BEA0-72BFDAAB2173}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
   <si>
     <t>Sets the capacity for batches of new installed capacity by technology. For updating assumptions by quantity of new capacity.</t>
   </si>
@@ -40,9 +40,6 @@
   </si>
   <si>
     <t>tech_generic</t>
-  </si>
-  <si>
-    <t>HYDRO_RUN</t>
   </si>
 </sst>
 </file>
@@ -360,7 +357,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K6"/>
+  <dimension ref="A1:K5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17.7109375" bestFit="1" customWidth="1"/>
@@ -481,41 +478,6 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>5</v>
-      </c>
-      <c r="B6">
-        <v>1000</v>
-      </c>
-      <c r="C6">
-        <v>1000</v>
-      </c>
-      <c r="D6">
-        <v>1000</v>
-      </c>
-      <c r="E6">
-        <v>1000</v>
-      </c>
-      <c r="F6">
-        <v>1000</v>
-      </c>
-      <c r="G6">
-        <v>1000</v>
-      </c>
-      <c r="H6">
-        <v>1000</v>
-      </c>
-      <c r="I6">
-        <v>1000</v>
-      </c>
-      <c r="J6">
-        <v>1000</v>
-      </c>
-      <c r="K6">
-        <v>1000</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
minor bug fix and scenario tinkering
</commit_message>
<xml_diff>
--- a/input_files/batched_new_capacity.xlsx
+++ b/input_files/batched_new_capacity.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://utoronto-my.sharepoint.com/personal/ian_elder_mail_utoronto_ca/Documents/Documents/TEMOA/CODERS scripts/input_files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="31" documentId="11_F25DC773A252ABDACC104858199A58E65ADE58E8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DB8E628F-AAAD-448E-BEA0-72BFDAAB2173}"/>
+  <xr:revisionPtr revIDLastSave="43" documentId="11_F25DC773A252ABDACC104858199A58E65ADE58E8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0C670D2A-6387-4B0F-8F29-E191BAB1AFEF}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2595" yWindow="885" windowWidth="21600" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ON" sheetId="1" r:id="rId1"/>
@@ -448,34 +448,34 @@
         <v>3</v>
       </c>
       <c r="B5">
-        <v>1000</v>
+        <v>2000</v>
       </c>
       <c r="C5">
-        <v>1000</v>
+        <v>2000</v>
       </c>
       <c r="D5">
-        <v>1000</v>
+        <v>2000</v>
       </c>
       <c r="E5">
-        <v>1000</v>
+        <v>2000</v>
       </c>
       <c r="F5">
-        <v>1000</v>
+        <v>2000</v>
       </c>
       <c r="G5">
-        <v>1000</v>
+        <v>2000</v>
       </c>
       <c r="H5">
-        <v>1000</v>
+        <v>2000</v>
       </c>
       <c r="I5">
-        <v>1000</v>
+        <v>2000</v>
       </c>
       <c r="J5">
-        <v>1000</v>
+        <v>2000</v>
       </c>
       <c r="K5">
-        <v>1000</v>
+        <v>2000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>